<commit_message>
Fix formula targets in Calc task 005 artifact
</commit_message>
<xml_diff>
--- a/evaluation_examples/expert_skill_learning/calc_full_v1/generated/round_01/artifacts/reference-task-calc-full-r01-005/initial_artifact.xlsx
+++ b/evaluation_examples/expert_skill_learning/calc_full_v1/generated/round_01/artifacts/reference-task-calc-full-r01-005/initial_artifact.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalog" sheetId="1" r:id="Rf52b7ffde1834681"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dispatch_Log" sheetId="2" r:id="R7f97e8761a5e45c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="Rdda6673fbbbb4864"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalog" sheetId="1" r:id="R2e2e0e280af041ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dispatch_Log" sheetId="2" r:id="Ra7a48b0a0d3748e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R44d481498691496b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -423,8 +423,8 @@
       <x:c r="D2" s="13" t="n">
         <x:v>238.5</x:v>
       </x:c>
-      <x:c r="E2" s="6"/>
-      <x:c r="F2" s="6"/>
+      <x:c r="E2" s="11"/>
+      <x:c r="F2" s="11"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="11" t="n">
@@ -439,8 +439,8 @@
       <x:c r="D3" s="13" t="n">
         <x:v>84</x:v>
       </x:c>
-      <x:c r="E3" s="6"/>
-      <x:c r="F3" s="6"/>
+      <x:c r="E3" s="11"/>
+      <x:c r="F3" s="11"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="11" t="n">
@@ -455,8 +455,8 @@
       <x:c r="D4" s="13" t="n">
         <x:v>416</x:v>
       </x:c>
-      <x:c r="E4" s="6"/>
-      <x:c r="F4" s="6"/>
+      <x:c r="E4" s="11"/>
+      <x:c r="F4" s="11"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="11" t="n">
@@ -471,8 +471,8 @@
       <x:c r="D5" s="13" t="n">
         <x:v>187.5</x:v>
       </x:c>
-      <x:c r="E5" s="6"/>
-      <x:c r="F5" s="6"/>
+      <x:c r="E5" s="11"/>
+      <x:c r="F5" s="11"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="11" t="n">
@@ -487,8 +487,8 @@
       <x:c r="D6" s="13" t="n">
         <x:v>135</x:v>
       </x:c>
-      <x:c r="E6" s="6"/>
-      <x:c r="F6" s="6"/>
+      <x:c r="E6" s="11"/>
+      <x:c r="F6" s="11"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="11" t="n">
@@ -503,8 +503,8 @@
       <x:c r="D7" s="13" t="n">
         <x:v>324</x:v>
       </x:c>
-      <x:c r="E7" s="6"/>
-      <x:c r="F7" s="6"/>
+      <x:c r="E7" s="11"/>
+      <x:c r="F7" s="11"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="11" t="n">
@@ -519,8 +519,8 @@
       <x:c r="D8" s="13" t="n">
         <x:v>270</x:v>
       </x:c>
-      <x:c r="E8" s="6"/>
-      <x:c r="F8" s="6"/>
+      <x:c r="E8" s="11"/>
+      <x:c r="F8" s="11"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="11" t="n">
@@ -535,8 +535,8 @@
       <x:c r="D9" s="13" t="n">
         <x:v>157.5</x:v>
       </x:c>
-      <x:c r="E9" s="6"/>
-      <x:c r="F9" s="6"/>
+      <x:c r="E9" s="11"/>
+      <x:c r="F9" s="11"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="11" t="n">
@@ -551,8 +551,8 @@
       <x:c r="D10" s="13" t="n">
         <x:v>56</x:v>
       </x:c>
-      <x:c r="E10" s="6"/>
-      <x:c r="F10" s="6"/>
+      <x:c r="E10" s="11"/>
+      <x:c r="F10" s="11"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="11" t="n">
@@ -567,8 +567,8 @@
       <x:c r="D11" s="13" t="n">
         <x:v>153</x:v>
       </x:c>
-      <x:c r="E11" s="6"/>
-      <x:c r="F11" s="6"/>
+      <x:c r="E11" s="11"/>
+      <x:c r="F11" s="11"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="11" t="n">
@@ -583,8 +583,8 @@
       <x:c r="D12" s="13" t="n">
         <x:v>180</x:v>
       </x:c>
-      <x:c r="E12" s="6"/>
-      <x:c r="F12" s="6"/>
+      <x:c r="E12" s="11"/>
+      <x:c r="F12" s="11"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="11" t="n">
@@ -599,8 +599,8 @@
       <x:c r="D13" s="13" t="n">
         <x:v>260</x:v>
       </x:c>
-      <x:c r="E13" s="6"/>
-      <x:c r="F13" s="6"/>
+      <x:c r="E13" s="11"/>
+      <x:c r="F13" s="11"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="11" t="n">
@@ -615,8 +615,8 @@
       <x:c r="D14" s="13" t="n">
         <x:v>225</x:v>
       </x:c>
-      <x:c r="E14" s="6"/>
-      <x:c r="F14" s="6"/>
+      <x:c r="E14" s="11"/>
+      <x:c r="F14" s="11"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="11" t="n">
@@ -631,8 +631,8 @@
       <x:c r="D15" s="13" t="n">
         <x:v>540</x:v>
       </x:c>
-      <x:c r="E15" s="6"/>
-      <x:c r="F15" s="6"/>
+      <x:c r="E15" s="11"/>
+      <x:c r="F15" s="11"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="11" t="n">
@@ -647,8 +647,8 @@
       <x:c r="D16" s="13" t="n">
         <x:v>150</x:v>
       </x:c>
-      <x:c r="E16" s="6"/>
-      <x:c r="F16" s="6"/>
+      <x:c r="E16" s="11"/>
+      <x:c r="F16" s="11"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="11" t="n">
@@ -663,8 +663,8 @@
       <x:c r="D17" s="13" t="n">
         <x:v>99</x:v>
       </x:c>
-      <x:c r="E17" s="6"/>
-      <x:c r="F17" s="6"/>
+      <x:c r="E17" s="11"/>
+      <x:c r="F17" s="11"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="11" t="n">
@@ -679,8 +679,8 @@
       <x:c r="D18" s="13" t="n">
         <x:v>272</x:v>
       </x:c>
-      <x:c r="E18" s="6"/>
-      <x:c r="F18" s="6"/>
+      <x:c r="E18" s="11"/>
+      <x:c r="F18" s="11"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="14" t="n">
@@ -695,8 +695,8 @@
       <x:c r="D19" s="16" t="n">
         <x:v>112.5</x:v>
       </x:c>
-      <x:c r="E19" s="7"/>
-      <x:c r="F19" s="7"/>
+      <x:c r="E19" s="14"/>
+      <x:c r="F19" s="14"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Fix Summary formula target in Calc task 005
</commit_message>
<xml_diff>
--- a/evaluation_examples/expert_skill_learning/calc_full_v1/generated/round_01/artifacts/reference-task-calc-full-r01-005/initial_artifact.xlsx
+++ b/evaluation_examples/expert_skill_learning/calc_full_v1/generated/round_01/artifacts/reference-task-calc-full-r01-005/initial_artifact.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalog" sheetId="1" r:id="R2e2e0e280af041ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dispatch_Log" sheetId="2" r:id="Ra7a48b0a0d3748e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R44d481498691496b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalog" sheetId="1" r:id="R0ef6a103700d4d44"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dispatch_Log" sheetId="2" r:id="R9930db5650a94f9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="Rfb02384af3d14131"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -723,87 +723,87 @@
       <x:c r="A2" s="6" t="str">
         <x:v>Total Units Dispatched</x:v>
       </x:c>
-      <x:c r="B2" s="6"/>
+      <x:c r="B2" s="11"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="6" t="str">
         <x:v>Review Note</x:v>
       </x:c>
-      <x:c r="B3" s="6" t="str">
+      <x:c r="B3" s="11" t="str">
         <x:v>Highest restock cost is flagged in Dispatch_Log</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="6"/>
-      <x:c r="B4" s="6"/>
+      <x:c r="B4" s="11"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="6"/>
-      <x:c r="B5" s="6"/>
+      <x:c r="B5" s="11"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="6"/>
-      <x:c r="B6" s="6"/>
+      <x:c r="B6" s="11"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="6"/>
-      <x:c r="B7" s="6"/>
+      <x:c r="B7" s="11"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="6"/>
-      <x:c r="B8" s="6"/>
+      <x:c r="B8" s="11"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="6"/>
-      <x:c r="B9" s="6"/>
+      <x:c r="B9" s="11"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="6"/>
-      <x:c r="B10" s="6"/>
+      <x:c r="B10" s="11"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="6"/>
-      <x:c r="B11" s="6"/>
+      <x:c r="B11" s="11"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="6"/>
-      <x:c r="B12" s="6"/>
+      <x:c r="B12" s="11"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="6"/>
-      <x:c r="B13" s="6"/>
+      <x:c r="B13" s="11"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="6"/>
-      <x:c r="B14" s="6"/>
+      <x:c r="B14" s="11"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="6"/>
-      <x:c r="B15" s="6"/>
+      <x:c r="B15" s="11"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="6"/>
-      <x:c r="B16" s="6"/>
+      <x:c r="B16" s="11"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="6"/>
-      <x:c r="B17" s="6"/>
+      <x:c r="B17" s="11"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="6"/>
-      <x:c r="B18" s="6"/>
+      <x:c r="B18" s="11"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="6"/>
-      <x:c r="B19" s="6"/>
+      <x:c r="B19" s="11"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="6"/>
-      <x:c r="B20" s="6"/>
+      <x:c r="B20" s="11"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="7"/>
-      <x:c r="B21" s="7"/>
+      <x:c r="B21" s="14"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>